<commit_message>
chore: fix rol/clases required in xlsx, merge onboarding docs into one
</commit_message>
<xml_diff>
--- a/docs/onboarding/Users_example.xlsx
+++ b/docs/onboarding/Users_example.xlsx
@@ -418,10 +418,10 @@
         <v>apellido</v>
       </c>
       <c r="D1" t="str">
-        <v>rol (opcional)</v>
+        <v>rol</v>
       </c>
       <c r="E1" t="str">
-        <v>clases (opcional)</v>
+        <v>clases</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Migration: Rol required, Precio/TipoPrecio/FechaInicio required, rename Clases->Asignaturas, group stat boxes
</commit_message>
<xml_diff>
--- a/docs/onboarding/Users_example.xlsx
+++ b/docs/onboarding/Users_example.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Usuarios" sheetId="1" r:id="rId1"/>
-    <sheet name="Clases" sheetId="2" r:id="rId2"/>
+    <sheet name="Asignaturas" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -421,7 +421,7 @@
         <v>rol</v>
       </c>
       <c r="E1" t="str">
-        <v>clases</v>
+        <v>asignaturas</v>
       </c>
     </row>
     <row r="2">
@@ -588,13 +588,13 @@
         <v>nombre</v>
       </c>
       <c r="B1" t="str">
-        <v>fechaInicio (opcional)</v>
+        <v>precio</v>
       </c>
       <c r="C1" t="str">
-        <v>precio (opcional)</v>
+        <v>tipoPrecio</v>
       </c>
       <c r="D1" t="str">
-        <v>tipoPrecio (opcional)</v>
+        <v>fechaInicio</v>
       </c>
       <c r="E1" t="str">
         <v>profesorEmail (opcional)</v>
@@ -620,13 +620,13 @@
         <v>Matemáticas 1</v>
       </c>
       <c r="B2" t="str">
+        <v>50</v>
+      </c>
+      <c r="C2" t="str">
+        <v>MENSUAL</v>
+      </c>
+      <c r="D2" t="str">
         <v>01/09/2026</v>
-      </c>
-      <c r="C2" t="str">
-        <v>50</v>
-      </c>
-      <c r="D2" t="str">
-        <v>MENSUAL</v>
       </c>
       <c r="E2" t="str">
         <v>miguel.ruiz@ejemplo.com</v>
@@ -652,13 +652,13 @@
         <v>Inglés B2</v>
       </c>
       <c r="B3" t="str">
+        <v>200</v>
+      </c>
+      <c r="C3" t="str">
+        <v>UNICO</v>
+      </c>
+      <c r="D3" t="str">
         <v>15/09/2026</v>
-      </c>
-      <c r="C3" t="str">
-        <v>200</v>
-      </c>
-      <c r="D3" t="str">
-        <v>UNICO</v>
       </c>
       <c r="E3" t="str">
         <v>sofia.moreno@ejemplo.com</v>
@@ -684,13 +684,13 @@
         <v>Ciencias</v>
       </c>
       <c r="B4" t="str">
+        <v>40</v>
+      </c>
+      <c r="C4" t="str">
+        <v>MENSUAL</v>
+      </c>
+      <c r="D4" t="str">
         <v>01/09/2026</v>
-      </c>
-      <c r="C4" t="str">
-        <v>40</v>
-      </c>
-      <c r="D4" t="str">
-        <v>MENSUAL</v>
       </c>
       <c r="E4" t="str">
         <v>sofia.moreno@ejemplo.com</v>

</xml_diff>

<commit_message>
fix: stripe payments excluded from pending table + implement pagado field + update migration docs
</commit_message>
<xml_diff>
--- a/docs/onboarding/Users_example.xlsx
+++ b/docs/onboarding/Users_example.xlsx
@@ -591,7 +591,7 @@
         <v>precio</v>
       </c>
       <c r="C1" t="str">
-        <v>tipoPrecio</v>
+        <v>cuotas (opcional)</v>
       </c>
       <c r="D1" t="str">
         <v>fechaInicio</v>
@@ -620,10 +620,10 @@
         <v>Matemáticas 1</v>
       </c>
       <c r="B2" t="str">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="C2" t="str">
-        <v>MENSUAL</v>
+        <v>10</v>
       </c>
       <c r="D2" t="str">
         <v>01/09/2026</v>
@@ -655,7 +655,7 @@
         <v>200</v>
       </c>
       <c r="C3" t="str">
-        <v>UNICO</v>
+        <v/>
       </c>
       <c r="D3" t="str">
         <v>15/09/2026</v>
@@ -684,10 +684,10 @@
         <v>Ciencias</v>
       </c>
       <c r="B4" t="str">
-        <v>40</v>
+        <v>400</v>
       </c>
       <c r="C4" t="str">
-        <v>MENSUAL</v>
+        <v>10</v>
       </c>
       <c r="D4" t="str">
         <v>01/09/2026</v>

</xml_diff>